<commit_message>
[Doc]: cập nhật bộ test report — Report 5.0, 5.1, 5.2, 5.2.2, 5.3, 5.4 sinh lại; testcase thủ công tách theo nhóm vào scripts/test_reports/cases (API và UI), thêm convert_xls.ps1, readable.py; cập nhật inventory, manifest, README và script sinh/kiểm tra report
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/08-reports/test-reports/Report5.3_System_Test.xlsx
+++ b/docs/08-reports/test-reports/Report5.3_System_Test.xlsx
@@ -1194,7 +1194,7 @@
         <v>Issue Date</v>
       </c>
       <c r="F5" s="14" t="str">
-        <v>2026-10-23</v>
+        <v>2026-10-29</v>
       </c>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
@@ -1222,8 +1222,8 @@
         <v>Document Code</v>
       </c>
       <c r="B6" s="16" t="str">
-        <f>B5&amp;"_"&amp;B2&amp;"_"&amp;F6</f>
-        <v>SEP490-G116_SYSTEM TEST REPORT DOCUMENT_1</v>
+        <f>B5&amp;"_"&amp;B2&amp;"_v"&amp;F6</f>
+        <v>SEP490-G116_SYSTEM TEST REPORT DOCUMENT_v1.1</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="6"/>
@@ -1231,7 +1231,7 @@
         <v>Version</v>
       </c>
       <c r="F6" s="17" t="str">
-        <v>1.0</v>
+        <v>1.1</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
@@ -1387,12 +1387,14 @@
       <c r="B11" s="26" t="str">
         <v>1.0</v>
       </c>
-      <c r="C11" s="27"/>
+      <c r="C11" s="27" t="str">
+        <v>Report 5</v>
+      </c>
       <c r="D11" s="28" t="str">
         <v>A</v>
       </c>
       <c r="E11" s="29" t="str">
-        <v>Generate English test documentation from TrustCabinet source using the supplied template.</v>
+        <v>Generate test documents from source</v>
       </c>
       <c r="F11" s="30"/>
       <c r="G11" s="31"/>
@@ -1417,12 +1419,22 @@
       <c r="Z11" s="31"/>
     </row>
     <row r="12" ht="21.75" customHeight="1">
-      <c r="A12" s="32"/>
-      <c r="B12" s="26"/>
-      <c r="C12" s="27"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="29"/>
-      <c r="F12" s="33"/>
+      <c r="A12" s="32" t="str">
+        <v>2026-10-29</v>
+      </c>
+      <c r="B12" s="26" t="str">
+        <v>1.1</v>
+      </c>
+      <c r="C12" s="27" t="str">
+        <v>Test cases</v>
+      </c>
+      <c r="D12" s="28" t="str">
+        <v>M</v>
+      </c>
+      <c r="E12" s="29" t="str">
+        <v>Regenerate: 1099 xUnit methods</v>
+      </c>
+      <c r="F12" s="33" t="str"/>
       <c r="G12" s="31"/>
       <c r="H12" s="31"/>
       <c r="I12" s="31"/>
@@ -1754,7 +1766,7 @@
         <v>Test requirement</v>
       </c>
       <c r="B3" s="103" t="str">
-        <v>Source-reviewed end-to-end workflow; record results only after execution.</v>
+        <v>System-level test flow: Isolate meeting data across roles</v>
       </c>
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
@@ -1794,7 +1806,7 @@
       <c r="N4" s="97"/>
       <c r="O4" s="99"/>
       <c r="P4" t="str">
-        <v>NotRun</v>
+        <v>Pending</v>
       </c>
     </row>
     <row r="5">
@@ -2009,7 +2021,7 @@
       <c r="O11" s="110"/>
       <c r="P11"/>
     </row>
-    <row r="12" ht="92" customHeight="1">
+    <row r="12" ht="109.5" customHeight="1">
       <c r="A12" s="108" t="str">
         <v>SYS-07</v>
       </c>
@@ -2019,23 +2031,19 @@
       <c r="C12" s="108" t="str">
         <v>1. Open list/details as each role.
 2. Try history, edit and transitions.
-3. Replace approver and retry as former
-approver.</v>
+3. Replace approver and retry as former approver.</v>
       </c>
       <c r="D12" s="108" t="str">
-        <v>Access follows relationship/state;
-unrelated or revoked users cannot read
-restricted data; inaccessible records
-return 404.</v>
+        <v>1. Access follows relationship/state.
+2. Unrelated or revoked users cannot read restricted data.
+3. Inaccessible records return 404.</v>
       </c>
       <c r="E12" s="108" t="str">
-        <v>Organizer, assigned approver,
-participant, outsider;
-Draft/WaitingApproval/Published
-fixtures.</v>
+        <v>1. Organizer, assigned approver, participant, outsider.
+2. Draft/WaitingApproval/Published fixtures.</v>
       </c>
       <c r="F12" s="108" t="str">
-        <v>NotRun</v>
+        <v>Pending</v>
       </c>
       <c r="G12" s="109" t="str"/>
       <c r="H12" s="108" t="str"/>
@@ -2045,11 +2053,7 @@
       <c r="L12" s="108" t="str"/>
       <c r="M12" s="109" t="str"/>
       <c r="N12" s="108" t="str"/>
-      <c r="O12" s="110" t="str">
-        <v>frontend/src/features/meeti
-ngs/detail/MeetingDetailPag
-e.tsx:1</v>
-      </c>
+      <c r="O12" s="110" t="str"/>
       <c r="P12"/>
     </row>
   </sheetData>
@@ -2131,7 +2135,7 @@
         <v>Test requirement</v>
       </c>
       <c r="B3" s="103" t="str">
-        <v>Source-reviewed end-to-end workflow; record results only after execution.</v>
+        <v>System-level test flow: Recover queued email after SMTP outage</v>
       </c>
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
@@ -2171,7 +2175,7 @@
       <c r="N4" s="97"/>
       <c r="O4" s="99"/>
       <c r="P4" t="str">
-        <v>NotRun</v>
+        <v>Pending</v>
       </c>
     </row>
     <row r="5">
@@ -2386,7 +2390,7 @@
       <c r="O11" s="110"/>
       <c r="P11"/>
     </row>
-    <row r="12" ht="110" customHeight="1">
+    <row r="12" ht="95.0" customHeight="1">
       <c r="A12" s="108" t="str">
         <v>SYS-08</v>
       </c>
@@ -2401,16 +2405,16 @@
 5. Compare mail and queue.</v>
       </c>
       <c r="D12" s="108" t="str">
-        <v>Publication persists; email retries
-after recovery without duplicate
-deduplication keys.</v>
+        <v>1. Publication persists.
+2. Email retries after recovery without duplicate deduplication keys.</v>
       </c>
       <c r="E12" s="108" t="str">
-        <v>Isolated staging; controllable SMTP
-sandbox; valid Approved fixture.</v>
+        <v>1. Isolated staging.
+2. Controllable SMTP sandbox.
+3. Valid Approved fixture.</v>
       </c>
       <c r="F12" s="108" t="str">
-        <v>NotRun</v>
+        <v>Pending</v>
       </c>
       <c r="G12" s="109" t="str"/>
       <c r="H12" s="108" t="str"/>
@@ -2420,11 +2424,7 @@
       <c r="L12" s="108" t="str"/>
       <c r="M12" s="109" t="str"/>
       <c r="N12" s="108" t="str"/>
-      <c r="O12" s="110" t="str">
-        <v>backend/TrustCabinet.Infras
-tructure/Email/EmailDeliver
-yWorker.cs:1</v>
-      </c>
+      <c r="O12" s="110" t="str"/>
       <c r="P12"/>
     </row>
   </sheetData>
@@ -2506,7 +2506,7 @@
         <v>Test requirement</v>
       </c>
       <c r="B3" s="103" t="str">
-        <v>Source-reviewed end-to-end workflow; record results only after execution.</v>
+        <v>System-level test flow: Operate agenda through complete meeting UI</v>
       </c>
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
@@ -2546,7 +2546,7 @@
       <c r="N4" s="97"/>
       <c r="O4" s="99"/>
       <c r="P4" t="str">
-        <v>NotRun</v>
+        <v>Pending</v>
       </c>
     </row>
     <row r="5">
@@ -2761,13 +2761,12 @@
       <c r="O11" s="110"/>
       <c r="P11"/>
     </row>
-    <row r="12" ht="92" customHeight="1">
+    <row r="12" ht="95.0" customHeight="1">
       <c r="A12" s="108" t="str">
         <v>SYS-09</v>
       </c>
       <c r="B12" s="108" t="str">
-        <v>Operate agenda through complete meeting
-UI</v>
+        <v>Operate agenda through complete meeting UI</v>
       </c>
       <c r="C12" s="108" t="str">
         <v>1. Create/reorder agenda in UI.
@@ -2776,16 +2775,14 @@
 4. Observe participant browser.</v>
       </c>
       <c r="D12" s="108" t="str">
-        <v>After integration, order/state/duration
-synchronize according to API; re-execute
-workflow.</v>
+        <v>1. After integration, order/state/duration synchronize according to API.
+2. Re-execute workflow.</v>
       </c>
       <c r="E12" s="108" t="str">
-        <v>Blocked: agenda UI and meeting-start
-workflow unavailable in this checkout.</v>
+        <v>1. Blocked: agenda UI and meeting-start workflow unavailable in this checkout.</v>
       </c>
       <c r="F12" s="108" t="str">
-        <v>Blocked</v>
+        <v>Pending</v>
       </c>
       <c r="G12" s="109" t="str"/>
       <c r="H12" s="108" t="str"/>
@@ -2795,11 +2792,7 @@
       <c r="L12" s="108" t="str"/>
       <c r="M12" s="109" t="str"/>
       <c r="N12" s="108" t="str"/>
-      <c r="O12" s="110" t="str">
-        <v>frontend/src/features/meeti
-ngs/detail/MeetingDetailPag
-e.tsx:1</v>
-      </c>
+      <c r="O12" s="110" t="str"/>
       <c r="P12"/>
     </row>
   </sheetData>
@@ -3076,7 +3069,7 @@
       <c r="Y8" s="51"/>
       <c r="Z8" s="51"/>
     </row>
-    <row r="9" ht="85" customHeight="1">
+    <row r="9" ht="80.5" customHeight="1">
       <c r="A9" s="10"/>
       <c r="B9" s="56" t="n">
         <v>1</v>
@@ -3091,7 +3084,10 @@
         <v>1 definitions / scenarios</v>
       </c>
       <c r="F9" s="59" t="str">
-        <v>AdminUsers; MeetingCreator role; new user; staging PostgreSQL/Redis.</v>
+        <v>1. AdminUsers.
+2. MeetingCreator role.
+3. New user.
+4. Staging PostgreSQL/Redis.</v>
       </c>
       <c r="G9" s="60"/>
       <c r="H9" s="10"/>
@@ -3114,7 +3110,7 @@
       <c r="Y9" s="10"/>
       <c r="Z9" s="10"/>
     </row>
-    <row r="10" ht="85" customHeight="1">
+    <row r="10" ht="66.0" customHeight="1">
       <c r="A10" s="10"/>
       <c r="B10" s="56" t="n">
         <v>2</v>
@@ -3129,7 +3125,9 @@
         <v>1 definitions / scenarios</v>
       </c>
       <c r="F10" s="59" t="str">
-        <v>Separate active organizer/approver; ready meeting; notification worker.</v>
+        <v>1. Separate active organizer/approver.
+2. Ready meeting.
+3. Notification worker.</v>
       </c>
       <c r="G10" s="60"/>
       <c r="H10" s="10"/>
@@ -3152,7 +3150,7 @@
       <c r="Y10" s="10"/>
       <c r="Z10" s="10"/>
     </row>
-    <row r="11" ht="85" customHeight="1">
+    <row r="11" ht="95.0" customHeight="1">
       <c r="A11" s="10"/>
       <c r="B11" s="56" t="n">
         <v>3</v>
@@ -3167,7 +3165,10 @@
         <v>1 definitions / scenarios</v>
       </c>
       <c r="F11" s="59" t="str">
-        <v>Approved fixture with active Chair/Secretary and participants; seeded roster; SMTP sandbox; workers enabled.</v>
+        <v>1. Approved fixture with active Chair/Secretary and participants.
+2. Seeded roster.
+3. SMTP sandbox.
+4. Workers enabled.</v>
       </c>
       <c r="G11" s="60"/>
       <c r="H11" s="10"/>
@@ -3190,7 +3191,7 @@
       <c r="Y11" s="10"/>
       <c r="Z11" s="10"/>
     </row>
-    <row r="12" ht="85" customHeight="1">
+    <row r="12" ht="80.5" customHeight="1">
       <c r="A12" s="10"/>
       <c r="B12" s="56" t="n">
         <v>4</v>
@@ -3205,7 +3206,10 @@
         <v>1 definitions / scenarios</v>
       </c>
       <c r="F12" s="59" t="str">
-        <v>Published meeting; participants; original invitation recorded; SMTP sandbox.</v>
+        <v>1. Published meeting.
+2. Participants.
+3. Original invitation recorded.
+4. SMTP sandbox.</v>
       </c>
       <c r="G12" s="60"/>
       <c r="H12" s="10"/>
@@ -3228,7 +3232,7 @@
       <c r="Y12" s="10"/>
       <c r="Z12" s="10"/>
     </row>
-    <row r="13" ht="85" customHeight="1">
+    <row r="13" ht="66.0" customHeight="1">
       <c r="A13" s="10"/>
       <c r="B13" s="56" t="n">
         <v>5</v>
@@ -3243,7 +3247,9 @@
         <v>1 definitions / scenarios</v>
       </c>
       <c r="F13" s="59" t="str">
-        <v>Independent admin; target signed in on two tabs; not final admin.</v>
+        <v>1. Independent admin.
+2. Target signed in on two tabs.
+3. Not final admin.</v>
       </c>
       <c r="G13" s="60"/>
       <c r="H13" s="10"/>
@@ -3266,7 +3272,7 @@
       <c r="Y13" s="10"/>
       <c r="Z13" s="10"/>
     </row>
-    <row r="14" ht="85" customHeight="1">
+    <row r="14" ht="66.0" customHeight="1">
       <c r="A14" s="10"/>
       <c r="B14" s="56" t="n">
         <v>6</v>
@@ -3281,7 +3287,9 @@
         <v>1 definitions / scenarios</v>
       </c>
       <c r="F14" s="59" t="str">
-        <v>Administrator/test user; SMTP sandbox; issued reset link.</v>
+        <v>1. Administrator/test user.
+2. SMTP sandbox.
+3. Issued reset link.</v>
       </c>
       <c r="G14" s="60"/>
       <c r="H14" s="10"/>
@@ -3304,7 +3312,7 @@
       <c r="Y14" s="10"/>
       <c r="Z14" s="10"/>
     </row>
-    <row r="15" ht="85" customHeight="1">
+    <row r="15" ht="80.5" customHeight="1">
       <c r="A15" s="10"/>
       <c r="B15" s="56" t="n">
         <v>7</v>
@@ -3319,7 +3327,8 @@
         <v>1 definitions / scenarios</v>
       </c>
       <c r="F15" s="59" t="str">
-        <v>Organizer, assigned approver, participant, outsider; Draft/WaitingApproval/Published fixtures.</v>
+        <v>1. Organizer, assigned approver, participant, outsider.
+2. Draft/WaitingApproval/Published fixtures.</v>
       </c>
       <c r="G15" s="60"/>
       <c r="H15" s="10"/>
@@ -3342,7 +3351,7 @@
       <c r="Y15" s="10"/>
       <c r="Z15" s="10"/>
     </row>
-    <row r="16" ht="85" customHeight="1">
+    <row r="16" ht="66.0" customHeight="1">
       <c r="A16" s="10"/>
       <c r="B16" s="56" t="n">
         <v>8</v>
@@ -3357,7 +3366,9 @@
         <v>1 definitions / scenarios</v>
       </c>
       <c r="F16" s="59" t="str">
-        <v>Isolated staging; controllable SMTP sandbox; valid Approved fixture.</v>
+        <v>1. Isolated staging.
+2. Controllable SMTP sandbox.
+3. Valid Approved fixture.</v>
       </c>
       <c r="G16" s="60"/>
       <c r="H16" s="10"/>
@@ -3380,7 +3391,7 @@
       <c r="Y16" s="10"/>
       <c r="Z16" s="10"/>
     </row>
-    <row r="17" ht="85" customHeight="1">
+    <row r="17" ht="51.5" customHeight="1">
       <c r="A17" s="10"/>
       <c r="B17" s="56" t="n">
         <v>9</v>
@@ -3395,7 +3406,7 @@
         <v>1 definitions / scenarios</v>
       </c>
       <c r="F17" s="59" t="str">
-        <v>Blocked: agenda UI and meeting-start workflow unavailable in this checkout.</v>
+        <v>1. Blocked: agenda UI and meeting-start workflow unavailable in this checkout.</v>
       </c>
       <c r="G17" s="60"/>
       <c r="H17" s="10"/>
@@ -3428,15 +3439,15 @@
     <mergeCell ref="D5:F5"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="D9" location="'WorkFlow1'!A1"/>
-    <hyperlink ref="D10" location="'WorkFlow2'!A1"/>
-    <hyperlink ref="D11" location="'WorkFlow3'!A1"/>
-    <hyperlink ref="D12" location="'WorkFlow4'!A1"/>
-    <hyperlink ref="D13" location="'WorkFlow5'!A1"/>
-    <hyperlink ref="D14" location="'WorkFlow6'!A1"/>
-    <hyperlink ref="D15" location="'WorkFlow7'!A1"/>
-    <hyperlink ref="D16" location="'WorkFlow8'!A1"/>
-    <hyperlink ref="D17" location="'WorkFlow9'!A1"/>
+    <hyperlink ref="D9" location="'WorkFlow1'!A1" display="WorkFlow1"/>
+    <hyperlink ref="D10" location="'WorkFlow2'!A1" display="WorkFlow2"/>
+    <hyperlink ref="D11" location="'WorkFlow3'!A1" display="WorkFlow3"/>
+    <hyperlink ref="D12" location="'WorkFlow4'!A1" display="WorkFlow4"/>
+    <hyperlink ref="D13" location="'WorkFlow5'!A1" display="WorkFlow5"/>
+    <hyperlink ref="D14" location="'WorkFlow6'!A1" display="WorkFlow6"/>
+    <hyperlink ref="D15" location="'WorkFlow7'!A1" display="WorkFlow7"/>
+    <hyperlink ref="D16" location="'WorkFlow8'!A1" display="WorkFlow8"/>
+    <hyperlink ref="D17" location="'WorkFlow9'!A1" display="WorkFlow9"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="1.1506944444444445" footer="0.0" header="0.0" left="0.7479166666666667" right="0.7479166666666667" top="0.9840277777777778"/>
@@ -3606,7 +3617,7 @@
       <c r="F5" s="6"/>
       <c r="G5" s="71"/>
       <c r="H5" s="76" t="str">
-        <v>2026-10-23</v>
+        <v>2026-10-29</v>
       </c>
       <c r="I5" s="10"/>
       <c r="J5" s="10"/>
@@ -3627,14 +3638,12 @@
       <c r="Y5" s="10"/>
       <c r="Z5" s="10"/>
     </row>
-    <row r="6" ht="60" customHeight="1">
+    <row r="6" ht="21.75" customHeight="1">
       <c r="A6" s="66"/>
       <c r="B6" s="74" t="str">
         <v>Notes</v>
       </c>
-      <c r="C6" s="77" t="str">
-        <v>Round 1. Pending: NotRun/Blocked/Partial. N/A: Skipped.</v>
-      </c>
+      <c r="C6" s="77" t="str"/>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
@@ -4345,15 +4354,15 @@
     <mergeCell ref="C6:H6"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C11" location="'WorkFlow1'!A1"/>
-    <hyperlink ref="C12" location="'WorkFlow2'!A1"/>
-    <hyperlink ref="C13" location="'WorkFlow3'!A1"/>
-    <hyperlink ref="C14" location="'WorkFlow4'!A1"/>
-    <hyperlink ref="C15" location="'WorkFlow5'!A1"/>
-    <hyperlink ref="C16" location="'WorkFlow6'!A1"/>
-    <hyperlink ref="C17" location="'WorkFlow7'!A1"/>
-    <hyperlink ref="C18" location="'WorkFlow8'!A1"/>
-    <hyperlink ref="C19" location="'WorkFlow9'!A1"/>
+    <hyperlink ref="C11" location="'WorkFlow1'!A1" display="WorkFlow1"/>
+    <hyperlink ref="C12" location="'WorkFlow2'!A1" display="WorkFlow2"/>
+    <hyperlink ref="C13" location="'WorkFlow3'!A1" display="WorkFlow3"/>
+    <hyperlink ref="C14" location="'WorkFlow4'!A1" display="WorkFlow4"/>
+    <hyperlink ref="C15" location="'WorkFlow5'!A1" display="WorkFlow5"/>
+    <hyperlink ref="C16" location="'WorkFlow6'!A1" display="WorkFlow6"/>
+    <hyperlink ref="C17" location="'WorkFlow7'!A1" display="WorkFlow7"/>
+    <hyperlink ref="C18" location="'WorkFlow8'!A1" display="WorkFlow8"/>
+    <hyperlink ref="C19" location="'WorkFlow9'!A1" display="WorkFlow9"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.9840277777777777" footer="0.0" header="0.0" left="0.7479166666666667" right="0.7479166666666667" top="0.9840277777777778"/>
@@ -4433,7 +4442,7 @@
         <v>Test requirement</v>
       </c>
       <c r="B3" s="103" t="str">
-        <v>Source-reviewed end-to-end workflow; record results only after execution.</v>
+        <v>System-level test flow: Provision access, create a meeting and revoke permission</v>
       </c>
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
@@ -4473,7 +4482,7 @@
       <c r="N4" s="97"/>
       <c r="O4" s="99"/>
       <c r="P4" t="str">
-        <v>NotRun</v>
+        <v>Pending</v>
       </c>
     </row>
     <row r="5">
@@ -4688,13 +4697,12 @@
       <c r="O11" s="110"/>
       <c r="P11"/>
     </row>
-    <row r="12" ht="110" customHeight="1">
+    <row r="12" ht="95.0" customHeight="1">
       <c r="A12" s="108" t="str">
         <v>SYS-01</v>
       </c>
       <c r="B12" s="108" t="str">
-        <v>Provision access, create a meeting and
-revoke permission</v>
+        <v>Provision access, create a meeting and revoke permission</v>
       </c>
       <c r="C12" s="108" t="str">
         <v>1. Create user and assign role.
@@ -4704,16 +4712,17 @@
 5. Reload and retry creation.</v>
       </c>
       <c r="D12" s="108" t="str">
-        <v>Creation succeeds while authorized and
-fails after revocation; original Draft
-remains intact.</v>
+        <v>1. Creation succeeds while authorized and fails after revocation.
+2. Original Draft remains intact.</v>
       </c>
       <c r="E12" s="108" t="str">
-        <v>AdminUsers; MeetingCreator role; new
-user; staging PostgreSQL/Redis.</v>
+        <v>1. AdminUsers.
+2. MeetingCreator role.
+3. New user.
+4. Staging PostgreSQL/Redis.</v>
       </c>
       <c r="F12" s="108" t="str">
-        <v>NotRun</v>
+        <v>Pending</v>
       </c>
       <c r="G12" s="109" t="str"/>
       <c r="H12" s="108" t="str"/>
@@ -4723,10 +4732,7 @@
       <c r="L12" s="108" t="str"/>
       <c r="M12" s="109" t="str"/>
       <c r="N12" s="108" t="str"/>
-      <c r="O12" s="110" t="str">
-        <v>frontend/src/features/acces
-s/UsersPage.tsx:1</v>
-      </c>
+      <c r="O12" s="110" t="str"/>
       <c r="P12"/>
     </row>
   </sheetData>
@@ -4808,7 +4814,7 @@
         <v>Test requirement</v>
       </c>
       <c r="B3" s="103" t="str">
-        <v>Source-reviewed end-to-end workflow; record results only after execution.</v>
+        <v>System-level test flow: Draft, submission, rejection, revision and approval</v>
       </c>
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
@@ -4848,7 +4854,7 @@
       <c r="N4" s="97"/>
       <c r="O4" s="99"/>
       <c r="P4" t="str">
-        <v>NotRun</v>
+        <v>Pending</v>
       </c>
     </row>
     <row r="5">
@@ -5063,33 +5069,32 @@
       <c r="O11" s="110"/>
       <c r="P11"/>
     </row>
-    <row r="12" ht="128" customHeight="1">
+    <row r="12" ht="95.0" customHeight="1">
       <c r="A12" s="108" t="str">
         <v>SYS-02</v>
       </c>
       <c r="B12" s="108" t="str">
-        <v>Draft, submission, rejection, revision
-and approval</v>
+        <v>Draft, submission, rejection, revision and approval</v>
       </c>
       <c r="C12" s="108" t="str">
         <v>1. Create and submit Draft.
-2. Read notification and reject with
-reason.
+2. Read notification and reject with reason.
 3. Revise and resubmit.
 4. Approve.
 5. Inspect history.</v>
       </c>
       <c r="D12" s="108" t="str">
-        <v>Transitions/recipients are correct;
-reasons and history persist;
-unauthorized actions fail.</v>
+        <v>1. Transitions/recipients are correct.
+2. Reasons and history persist.
+3. Unauthorized actions fail.</v>
       </c>
       <c r="E12" s="108" t="str">
-        <v>Separate active organizer/approver;
-ready meeting; notification worker.</v>
+        <v>1. Separate active organizer/approver.
+2. Ready meeting.
+3. Notification worker.</v>
       </c>
       <c r="F12" s="108" t="str">
-        <v>NotRun</v>
+        <v>Pending</v>
       </c>
       <c r="G12" s="109" t="str"/>
       <c r="H12" s="108" t="str"/>
@@ -5099,11 +5104,7 @@
       <c r="L12" s="108" t="str"/>
       <c r="M12" s="109" t="str"/>
       <c r="N12" s="108" t="str"/>
-      <c r="O12" s="110" t="str">
-        <v>frontend/src/features/meeti
-ngs/workflow/MeetingWorkflo
-wBar.tsx:1</v>
-      </c>
+      <c r="O12" s="110" t="str"/>
       <c r="P12"/>
     </row>
   </sheetData>
@@ -5185,7 +5186,7 @@
         <v>Test requirement</v>
       </c>
       <c r="B3" s="103" t="str">
-        <v>Source-reviewed end-to-end workflow; record results only after execution.</v>
+        <v>System-level test flow: Publication, notifications, email and Calendar</v>
       </c>
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
@@ -5225,7 +5226,7 @@
       <c r="N4" s="97"/>
       <c r="O4" s="99"/>
       <c r="P4" t="str">
-        <v>NotRun</v>
+        <v>Pending</v>
       </c>
     </row>
     <row r="5">
@@ -5440,13 +5441,12 @@
       <c r="O11" s="110"/>
       <c r="P11"/>
     </row>
-    <row r="12" ht="92" customHeight="1">
+    <row r="12" ht="124.0" customHeight="1">
       <c r="A12" s="108" t="str">
         <v>SYS-03</v>
       </c>
       <c r="B12" s="108" t="str">
-        <v>Publication, notifications, email and
-Calendar</v>
+        <v>Publication, notifications, email and Calendar</v>
       </c>
       <c r="C12" s="108" t="str">
         <v>1. Publish.
@@ -5455,18 +5455,19 @@
 4. Compare Calendar and details.</v>
       </c>
       <c r="D12" s="108" t="str">
-        <v>Published status and schedule agree;
-intended recipients receive invitation;
-retries do not duplicate; outsiders
-receive no data.</v>
+        <v>1. Published status and schedule agree.
+2. Intended recipients receive invitation.
+3. Retries do not duplicate.
+4. Outsiders receive no data.</v>
       </c>
       <c r="E12" s="108" t="str">
-        <v>Approved fixture with active
-Chair/Secretary and participants; seeded
-roster; SMTP sandbox; workers enabled.</v>
+        <v>1. Approved fixture with active Chair/Secretary and participants.
+2. Seeded roster.
+3. SMTP sandbox.
+4. Workers enabled.</v>
       </c>
       <c r="F12" s="108" t="str">
-        <v>NotRun</v>
+        <v>Pending</v>
       </c>
       <c r="G12" s="109" t="str"/>
       <c r="H12" s="108" t="str"/>
@@ -5476,11 +5477,7 @@
       <c r="L12" s="108" t="str"/>
       <c r="M12" s="109" t="str"/>
       <c r="N12" s="108" t="str"/>
-      <c r="O12" s="110" t="str">
-        <v>frontend/src/features/meeti
-ngs/workflow/MeetingWorkflo
-wBar.tsx:1</v>
-      </c>
+      <c r="O12" s="110" t="str"/>
       <c r="P12"/>
     </row>
   </sheetData>
@@ -5562,7 +5559,7 @@
         <v>Test requirement</v>
       </c>
       <c r="B3" s="103" t="str">
-        <v>Source-reviewed end-to-end workflow; record results only after execution.</v>
+        <v>System-level test flow: Synchronize published meeting reschedule</v>
       </c>
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
@@ -5602,7 +5599,7 @@
       <c r="N4" s="97"/>
       <c r="O4" s="99"/>
       <c r="P4" t="str">
-        <v>NotRun</v>
+        <v>Pending</v>
       </c>
     </row>
     <row r="5">
@@ -5817,7 +5814,7 @@
       <c r="O11" s="110"/>
       <c r="P11"/>
     </row>
-    <row r="12" ht="110" customHeight="1">
+    <row r="12" ht="95.0" customHeight="1">
       <c r="A12" s="108" t="str">
         <v>SYS-04</v>
       </c>
@@ -5827,22 +5824,22 @@
       <c r="C12" s="108" t="str">
         <v>1. Reschedule.
 2. Inspect history.
-3. Check bell, update email and
-Calendar.
+3. Check bell, update email and Calendar.
 4. Reload both browsers.</v>
       </c>
       <c r="D12" s="108" t="str">
-        <v>All screens show latest schedule;
-history records change; updates contain
-new time.</v>
+        <v>1. All screens show latest schedule.
+2. History records change.
+3. Updates contain new time.</v>
       </c>
       <c r="E12" s="108" t="str">
-        <v>Published meeting; participants;
-original invitation recorded; SMTP
-sandbox.</v>
+        <v>1. Published meeting.
+2. Participants.
+3. Original invitation recorded.
+4. SMTP sandbox.</v>
       </c>
       <c r="F12" s="108" t="str">
-        <v>NotRun</v>
+        <v>Pending</v>
       </c>
       <c r="G12" s="109" t="str"/>
       <c r="H12" s="108" t="str"/>
@@ -5852,10 +5849,7 @@
       <c r="L12" s="108" t="str"/>
       <c r="M12" s="109" t="str"/>
       <c r="N12" s="108" t="str"/>
-      <c r="O12" s="110" t="str">
-        <v>frontend/src/features/meeti
-ngs/MeetingForm.tsx:1</v>
-      </c>
+      <c r="O12" s="110" t="str"/>
       <c r="P12"/>
     </row>
   </sheetData>
@@ -5937,7 +5931,7 @@
         <v>Test requirement</v>
       </c>
       <c r="B3" s="103" t="str">
-        <v>Source-reviewed end-to-end workflow; record results only after execution.</v>
+        <v>System-level test flow: Deactivate, revoke sessions and restore access</v>
       </c>
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
@@ -5977,7 +5971,7 @@
       <c r="N4" s="97"/>
       <c r="O4" s="99"/>
       <c r="P4" t="str">
-        <v>NotRun</v>
+        <v>Pending</v>
       </c>
     </row>
     <row r="5">
@@ -6192,13 +6186,12 @@
       <c r="O11" s="110"/>
       <c r="P11"/>
     </row>
-    <row r="12" ht="92" customHeight="1">
+    <row r="12" ht="109.5" customHeight="1">
       <c r="A12" s="108" t="str">
         <v>SYS-05</v>
       </c>
       <c r="B12" s="108" t="str">
-        <v>Deactivate, revoke sessions and restore
-access</v>
+        <v>Deactivate, revoke sessions and restore access</v>
       </c>
       <c r="C12" s="108" t="str">
         <v>1. Deactivate target.
@@ -6207,17 +6200,17 @@
 4. Sign in again.</v>
       </c>
       <c r="D12" s="108" t="str">
-        <v>Operations fail while inactive; new
-sign-in succeeds after reactivation; old
-sessions cannot bypass active-user
-checks.</v>
+        <v>1. Operations fail while inactive.
+2. New sign-in succeeds after reactivation.
+3. Old sessions cannot bypass active-user checks.</v>
       </c>
       <c r="E12" s="108" t="str">
-        <v>Independent admin; target signed in on
-two tabs; not final admin.</v>
+        <v>1. Independent admin.
+2. Target signed in on two tabs.
+3. Not final admin.</v>
       </c>
       <c r="F12" s="108" t="str">
-        <v>NotRun</v>
+        <v>Pending</v>
       </c>
       <c r="G12" s="109" t="str"/>
       <c r="H12" s="108" t="str"/>
@@ -6227,10 +6220,7 @@
       <c r="L12" s="108" t="str"/>
       <c r="M12" s="109" t="str"/>
       <c r="N12" s="108" t="str"/>
-      <c r="O12" s="110" t="str">
-        <v>frontend/src/features/acces
-s/UsersPage.tsx:1</v>
-      </c>
+      <c r="O12" s="110" t="str"/>
       <c r="P12"/>
     </row>
   </sheetData>
@@ -6312,7 +6302,7 @@
         <v>Test requirement</v>
       </c>
       <c r="B3" s="103" t="str">
-        <v>Source-reviewed end-to-end workflow; record results only after execution.</v>
+        <v>System-level test flow: Reset password across email and authentication</v>
       </c>
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
@@ -6352,7 +6342,7 @@
       <c r="N4" s="97"/>
       <c r="O4" s="99"/>
       <c r="P4" t="str">
-        <v>NotRun</v>
+        <v>Pending</v>
       </c>
     </row>
     <row r="5">
@@ -6567,33 +6557,33 @@
       <c r="O11" s="110"/>
       <c r="P11"/>
     </row>
-    <row r="12" ht="128" customHeight="1">
+    <row r="12" ht="95.0" customHeight="1">
       <c r="A12" s="108" t="str">
         <v>SYS-06</v>
       </c>
       <c r="B12" s="108" t="str">
-        <v>Reset password across email and
-authentication</v>
+        <v>Reset password across email and authentication</v>
       </c>
       <c r="C12" s="108" t="str">
         <v>1. Request reset.
 2. Complete through email.
 3. Try old/new passwords.
 4. Reuse token.
-5. Check old sessions against auth
-contract.</v>
+5. Check old sessions against auth contract.</v>
       </c>
       <c r="D12" s="108" t="str">
-        <v>Old password fails; new one works; token
-is single-use; session revocation
-follows backend contract.</v>
+        <v>1. Old password fails.
+2. New one works.
+3. Token is single-use.
+4. Session revocation follows backend contract.</v>
       </c>
       <c r="E12" s="108" t="str">
-        <v>Administrator/test user; SMTP sandbox;
-issued reset link.</v>
+        <v>1. Administrator/test user.
+2. SMTP sandbox.
+3. Issued reset link.</v>
       </c>
       <c r="F12" s="108" t="str">
-        <v>NotRun</v>
+        <v>Pending</v>
       </c>
       <c r="G12" s="109" t="str"/>
       <c r="H12" s="108" t="str"/>
@@ -6603,10 +6593,7 @@
       <c r="L12" s="108" t="str"/>
       <c r="M12" s="109" t="str"/>
       <c r="N12" s="108" t="str"/>
-      <c r="O12" s="110" t="str">
-        <v>frontend/src/features/auth/
-LoginPage.tsx:1</v>
-      </c>
+      <c r="O12" s="110" t="str"/>
       <c r="P12"/>
     </row>
   </sheetData>

</xml_diff>